<commit_message>
feat(chowchow): replenish 31 verified dog products, enforce dog-only filter, and enhance review logging
</commit_message>
<xml_diff>
--- a/review_products.xlsx
+++ b/review_products.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="630" yWindow="615" windowWidth="37095" windowHeight="17310" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Products" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="posted_state" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="posted_state" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G173"/>
+  <dimension ref="A1:G204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4960,6 +4960,781 @@
       <c r="G173" t="inlineStr">
         <is>
           <t>done 2026-08-02 19:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="n">
+        <v>147</v>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>PANDO Pet Dryer Room PD65 แพนโด้ เครื่องเป่าขน สำหรับสัตว์เลี้ยง รุ่น PD65 ตู้เป่าขน อัตโนม</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/2qRzC0bKNG</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztm-mp1zyxmcgm4r44.webp</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>฿9990.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="n">
+        <v>148</v>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>พร้อมส่ง MJ.Kudson อาหารสุนัขพรีเมียมสูตรแกะ (ลดขนร่วง ลดคราบน้ำตา ลดกลิ่นมูลสัตว์) ทานได้ทุกสายพันธุ์</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/4AxMmSnMyM</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zto-mopbxox2cfm73f.webp</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>฿547.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="n">
+        <v>149</v>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Dr.Zkin Pet Spray ผลิตภัณฑ์สำหรับสัตว์เลี้ยง บำรุงขน ดับกลิ่น เพิ่มความหอม</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/70HY9gQhNc</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztg-mhh7zikraarne4.webp</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>฿210.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="n">
+        <v>150</v>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Prowild โปรไวลด์ ซีเล็คเต็ด อาหารสุนัขทุกสายพันธุ์/ทุกช่วงวัย ขนาด 15 kg</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/9fIJKaWMHK</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0m-mbg6gn8vi82g66.webp</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>฿1590.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="n">
+        <v>151</v>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>NaviPet Grooming Vacuum KIT 7 in 1 เครื่องปัตตาเลียนตัดแต่งขนสำหรับสัตว์เลี้ยง และดูดฝุ่น กรูมมิ่งสำหรับดูด</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/40e06K2cCJ</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasc-madx77cb5x8wff.webp</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>฿2590.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="n">
+        <v>152</v>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>PANDO Second Generation Pet Trolleyแพนโด้ รถเข็นสำหรับสัตว์เลี้ยง เวอร์ชันอัพเกรด</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/110OWov8hV</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztg-mp208h070r2883.webp</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>฿3390.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="n">
+        <v>153</v>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>navipet Smart Pet Dryer (Thai Version) ตู้เป่า ขนสัตว์เลี้ยง 72ลิตร O ZONE ฆ่าเชื้อได้ ประกันศูนย์ไทย</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/6pyBTXqfWJ</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztn-mnqj2jpnw45hd8.webp</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>฿7900.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="n">
+        <v>154</v>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>แนะนำ! สมาร์ทฮาร์ท โกลด์ ฟิตแอนด์เฟิร์ม 7+ อาหารสุนัขสูงอายุ พันธุ์กลาง-ใหญ่ 20 กก.</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/9pbn350qIc</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztp-mp3d3pouixhqeb.webp</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>฿1480.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="n">
+        <v>155</v>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>[สินค้าใหม่] PANDO Pet Hair Trimmer 4 in 1 Pro แพนโด้ ชุดอุปกรณ์ตัดขน เล็มขน สัตว์เลี้ยง รุ่น โปร</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/30lSuWWyVO</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zto-mp20bnax2bkd6b.webp</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>฿581.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="n">
+        <v>156</v>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Pawdy อาหารสุนัขเกรดพรีเมียม Holistic สำหรับสุนัขโต อายุ 1-6 ปี สูตรเนื้อแกะรมควัน ขนาด 8 กก.</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/9pbn35XQb1</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zth-mn700alam03s8d.webp</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>฿1359.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="n">
+        <v>157</v>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>พร้อมส่ง MJ.Kudson อาหารสุนัขพรีเมียมสูตรแกะ (ลดขนร่วง ลดคราบน้ำตา ลดกลิ่นมูลสัตว์) ทานได้ทุกสายพันธุ์</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/W47vxAxHm</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zto-mopbxox2cfm73f.webp</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>฿547.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="n">
+        <v>158</v>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>[Doctor By BREATH CARE] อาหารเสริมทางเดินหายใจสุนัข บรรเทาอาการไอ ฮอนคิง แก้สงสารพยุงบรอนเชียล (30 บีบ)</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/8KmzGMOid3</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/sg-11134207-822wp-mog5oph3ouml25.webp</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>฿1126.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="n">
+        <v>159</v>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>[ ตกกิโลละ 119 บาท l ไซส์กระสอบ 15 กิโล ] petheria อาหารสุนัขแบบเม็ดเกรด SUPER PREMIUM มีให้เลือกทุกช่วงวัย</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/70HbfvolrB</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98w-lwv3eh1w2dan86.webp</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>฿1798.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="n">
+        <v>160</v>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Dog Days อาหารลูกสุนัข (6 kg) สูตร Puppy &amp; Mommy รสแกะและปลาทูน่า</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/110OWujz86</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zth-modfibxbvymma0.webp</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>฿690.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="n">
+        <v>161</v>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Dog Days อาหารสุนัขรสเนื้อแกะ (12 kg) Daily เกรด Holistic สูตรลดขนร่วงโดยเฉพาะ โซเดียมต่ำ</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/8fPpf2BSBB</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zth-mp3judrlwkcr9c.webp</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>฿1691.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="n">
+        <v>162</v>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Petcho แผ่นรองฉี่ แผ่นรองฉี่สุนัข แผ่นรองซับ สัตว์เลี้ยง ซับได้มาก พลังการดูดซับ 6ชั้น ช่วยฝึกขับถ่าย</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/W47w2T99w</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r98t-lyelrzpqov41c6.webp</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>฿149.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="n">
+        <v>163</v>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>เสื้อน้องหมาลาย เครื่องปรุงรส ผ้าไมโครสีสันสดใสพร้อมส่ง</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/6pyBTgRAjL</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasa-m96tiq9mlglrc3.webp</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>฿50.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="n">
+        <v>164</v>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>NAVIPET Wireless Drinking Fountain V1 น้ำพุไร้สายความจุ2.5ลิตร มีแบตในตัว5000 mAh ประกันศูนย์ไทย1 ปี</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/gNY8M5yK7</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztj-mf998jaiwff3bb.webp</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>฿742.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="n">
+        <v>165</v>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Pawdy อาหารสุนัขเกรดพรีเมียม สำหรับสุนัขสูงวัย อายุมากกว่า 7 ปี สูตรแกะและปลา ผสมเนื้อจระเข้ ขนาด 1.2 กก.</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/4LGqV615Un</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztk-mn9tb9drwvszd2.webp</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>฿333.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="n">
+        <v>166</v>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Prama อาหารสุนัขพราม่าเกรด Holistic มีให้เลือก 2 สูตร เนื้อแกะ และ ปลาทูน่า ขนาด 15kg</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/9Uywec7H9V</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasa-m2idzdnzkn8k02.webp</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>฿1250.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="n">
+        <v>167</v>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Pawdy อาหารสุนัขเกรดพรีเมียม สำหรับสุนัขสูงวัย อายุมากกว่า 7 ปี สูตรแกะและปลา ผสมเนื้อจระเข้ ขนาด 1.2 กก. (2 ถุง)</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/4qD763Stp2</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztg-mkgeybc3sfewa9.webp</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>฿643.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="n">
+        <v>168</v>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>PANDO Pet Smart Camera Feeder 4L เครื่องให้อาหารอัตโนมัติขนาด 4 ลิตร พร้อมกล้องวิดีโอ</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/AUrTqTY04A</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zte-mp20hqahb9xq74.webp</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>฿3790.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="n">
+        <v>169</v>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>My Paws น้ำยาล้างจาน น้ำยาล้างของเล่น น้ำยาล้างจานสำหรับสัตว์เลี้ยง สารสกัดจากธรรมชาติ อ่อนโยน สำหรับสัตว์เลี้ยงทุกชนิด</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/1Vwf7wPVkj</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztc-mp37aagvwj5te3.webp</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>฿38.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="n">
+        <v>170</v>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Pawdy อาหารสุนัขเกรดพรีเมียม Holistic สำหรับสุนัขโต อายุ 1-6 ปี สูตรเนื้อวัวย่างและเห็ดทรัฟเฟิล ขนาด 8 กก. (มี 2 ขนาด)</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/8ATZ4DLj5r</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztm-mn6zvfws7coy54.webp</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>฿1278.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="n">
+        <v>171</v>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>yoyopet : แปรงกําจัดขนสองด้าน แปรงสางขนเสีย หวีซี่สแตนเลส กำจัดขนลอย ขนปม อุปกรณ์ดูแลขนสัตว์เลี้ยง</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/7fXITJ3q7F</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasm-m4ze403ouvtpc2.webp</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>฿58.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="n">
+        <v>172</v>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>สมาร์ทฮาร์ท อาหารสุนัข สำหรับลูกสุนัข รสเนื้อวัวและนม 15กก.</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/gNY8RukUK</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/9ec893796776a5020ab0abee60620b57.webp</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>฿1030.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="n">
+        <v>173</v>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>(คละรสไม่ได้) สมาร์ทฮาร์ท อาหารสุนัขกระป๋อง 400g x24 กระป๋อง(ยกแพ็ค)</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/9KfWSNx5gi</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81zth-mlx53j8akmbp86.webp</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>฿1090.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="n">
+        <v>174</v>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>PANDO Double-Layer Pet Trolley แพนโด้ รถเข็นแบบสองชั้นสำหรับสัตว์เลี้ยง</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/40e06ahvjJ</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-81ztm-mj6sg1hg00sj92.webp</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>฿5990.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="n">
+        <v>175</v>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>[ขายดี] สมาร์ทฮาร์ท อาหารสุนัข สุนัขโต รสเนื้ออบ 10 กก. / SmartHeart Adult Roast Beef 10kg</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/70Hbg6gXva</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7rasd-m682zid86p6f5f.webp</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>฿819.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="n">
+        <v>176</v>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>[แบรนด์ขายดีอันดับ 1]JerHigh เจอร์ไฮ สติ๊ก ขนมสุนัข ขนาด 60 กรัม จำนวน 12 ซอง (เลือกรสด้านใน)</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/7VDsH33sg7</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7ra0s-mb7mtm884ks64b.webp</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>฿741.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="n">
+        <v>177</v>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>กรง สแตนเลส 304 กรงสัตว์เลี้ยงขนาดใหญ่（125*110cm）กรงสแตนเลส กรงสุนัขพับได้ กรงสุนัข คอกกรงสัตว์เลี้ยง dog cages crates</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/qgyKnqQa2</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>https://down-bs-th.img.susercontent.com/th-11134207-7r992-lya8q6n2fnah9e.webp</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>฿2667.00</t>
         </is>
       </c>
     </row>

</xml_diff>